<commit_message>
Update roster: Export Roster June 2026 Version3.xlsx
</commit_message>
<xml_diff>
--- a/rosters/.versions/2026-06/current.xlsx
+++ b/rosters/.versions/2026-06/current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omanair-my.sharepoint.com/personal/80235_hq_omanair_com/Documents/Desktop/Rosters/STAFF OPERATION SCHEDULE/Roster with 2 OFF/05June/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE75BAC3-01A8-4F4B-A53B-0B41260E82E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{CE75BAC3-01A8-4F4B-A53B-0B41260E82E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88B5E81A-A54C-44CD-A4F6-4E91E1F258F6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{9736B67C-D61B-41E1-B07B-429B3D8AE9CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="4" xr2:uid="{9736B67C-D61B-41E1-B07B-429B3D8AE9CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Setting " sheetId="1" state="hidden" r:id="rId1"/>
@@ -35689,13 +35689,13 @@
         <v>231</v>
       </c>
       <c r="I16" s="84" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J16" s="84" t="s">
         <v>230</v>
       </c>
       <c r="K16" s="84" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="L16" s="84" t="s">
         <v>234</v>
@@ -35780,11 +35780,11 @@
       </c>
       <c r="AN16" s="48">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO16" s="48">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP16" s="48">
         <f t="shared" si="4"/>
@@ -37240,7 +37240,7 @@
       </c>
       <c r="D29" s="107"/>
       <c r="F29" s="84" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="G29" s="84" t="s">
         <v>215</v>
@@ -37344,7 +37344,7 @@
       </c>
       <c r="AO29" s="48">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AP29" s="48">
         <f t="shared" si="4"/>
@@ -37966,19 +37966,19 @@
         <v>215</v>
       </c>
       <c r="H35" s="84" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="I35" s="84" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="J35" s="84" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="K35" s="84" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="L35" s="84" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="M35" s="84" t="s">
         <v>215</v>
@@ -38056,11 +38056,11 @@
       </c>
       <c r="AM35" s="48">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AN35" s="48">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AO35" s="48">
         <f t="shared" si="3"/>
@@ -38200,13 +38200,13 @@
       </c>
       <c r="D37" s="117"/>
       <c r="F37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="G37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="H37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="I37" s="174" t="s">
         <v>126</v>
@@ -38221,13 +38221,13 @@
         <v>215</v>
       </c>
       <c r="M37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="N37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="O37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="P37" s="174" t="s">
         <v>231</v>
@@ -38242,13 +38242,13 @@
         <v>215</v>
       </c>
       <c r="T37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="U37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="V37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="W37" s="174" t="s">
         <v>231</v>
@@ -38284,10 +38284,10 @@
         <v>215</v>
       </c>
       <c r="AH37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="AI37" s="174" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="AJ37" s="174"/>
       <c r="AL37" s="48">
@@ -38365,11 +38365,11 @@
       </c>
       <c r="I39" s="37">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J39" s="37">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K39" s="37">
         <f t="shared" si="5"/>
@@ -38377,7 +38377,7 @@
       </c>
       <c r="L39" s="37">
         <f t="shared" si="5"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M39" s="37">
         <f t="shared" si="5"/>
@@ -38492,7 +38492,7 @@
       </c>
       <c r="H40" s="37">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I40" s="37">
         <f t="shared" si="6"/>
@@ -38615,7 +38615,7 @@
       <c r="E41" s="36"/>
       <c r="F41" s="37">
         <f t="shared" ref="F41:AJ41" si="7">COUNTIF(F$5:F$36,"N*")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G41" s="37">
         <f t="shared" si="7"/>
@@ -38635,7 +38635,7 @@
       </c>
       <c r="K41" s="37">
         <f t="shared" si="7"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L41" s="37">
         <f t="shared" si="7"/>
@@ -39139,7 +39139,7 @@
       <c r="E45" s="38"/>
       <c r="F45" s="50">
         <f>F47-F48</f>
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="G45" s="50">
         <f t="shared" ref="G45:AJ45" si="11">G47-G48</f>
@@ -39147,23 +39147,23 @@
       </c>
       <c r="H45" s="50">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I45" s="50">
         <f t="shared" si="11"/>
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="J45" s="50">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K45" s="50">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L45" s="50">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M45" s="50">
         <f t="shared" si="11"/>
@@ -39306,7 +39306,7 @@
       <c r="E47" s="36"/>
       <c r="F47" s="41">
         <f>SUM(F39:F41)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G47" s="41">
         <f t="shared" ref="G47:AI47" si="12">SUM(G39:G41)</f>
@@ -39314,23 +39314,23 @@
       </c>
       <c r="H47" s="41">
         <f t="shared" si="12"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I47" s="41">
         <f t="shared" si="12"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J47" s="41">
         <f t="shared" si="12"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K47" s="41">
         <f t="shared" si="12"/>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L47" s="41">
         <f t="shared" si="12"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M47" s="41">
         <f t="shared" si="12"/>
@@ -39536,7 +39536,7 @@
       <c r="E49" s="36"/>
       <c r="F49" s="37">
         <f>SUM(F39,F40,F41,F42,F44)</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G49" s="37">
         <f t="shared" ref="G49:AI49" si="13">SUM(G39,G40,G41,G42,G44)</f>
@@ -39544,23 +39544,23 @@
       </c>
       <c r="H49" s="37">
         <f t="shared" si="13"/>
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I49" s="37">
         <f t="shared" si="13"/>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J49" s="37">
         <f t="shared" si="13"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K49" s="37">
         <f t="shared" si="13"/>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L49" s="37">
         <f t="shared" si="13"/>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M49" s="37">
         <f t="shared" si="13"/>

</xml_diff>